<commit_message>
Add renewable energy cost per unit column to the time series
Adds a per-year renewable cost per unit alongside the blended rate on the
Time Series tab, and an FY25 weighted row on the Source Rates tab to
support it.

For FY05 to FY14 the renewable rate is the units-weighted blend of the
solar and wind lines in Form A, which appear only from FY13; earlier
years show a dash because no renewable capacity was reported. FY25 and
FY26 come from the renewable line of the quarterly power mix tables,
weighted by quarterly units. FY24 is not available because the FY24 decks
publish no source-wise split.

Also corrects the units formula on the modern block, which still pointed
at the pre-insertion volume column and silently produced wrong values for
FY25 and FY26 while only erroring on FY24.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ce8uyL4yMXyavjjecjxHpc
</commit_message>
<xml_diff>
--- a/out/UltraTech_Electricity_Cost_Timeseries.xlsx
+++ b/out/UltraTech_Electricity_Cost_Timeseries.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="145">
   <si>
     <t xml:space="preserve">ULTRATECH CEMENT — ELECTRICITY COST TIME SERIES</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">Blended cost (Rs./kWh)</t>
   </si>
   <si>
+    <t xml:space="preserve">Renewable energy cost (Rs./kWh)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cement volume (MnT)</t>
   </si>
   <si>
@@ -356,6 +359,9 @@
   </si>
   <si>
     <t xml:space="preserve">Q4FY26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25 weighted (Q2-Q4 only)</t>
   </si>
   <si>
     <t xml:space="preserve">FY26 weighted</t>
@@ -638,7 +644,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -692,6 +698,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1043,16 +1053,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1101,10 +1112,13 @@
       <c r="J5" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="K5" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1115,10 +1129,11 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">(Workings!B6*Workings!C6+Workings!D6*Workings!E6+Workings!F6*Workings!G6+Workings!H6*Workings!I6+Workings!J6*Workings!K6+Workings!L6*Workings!M6+Workings!N6*Workings!O6)*1000/10000000</f>
@@ -1144,15 +1159,19 @@
         <f aca="false">B7*10000000/(F7*1000000)</f>
         <v>3.41291939368347</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L6*Workings!M6+Workings!N6*Workings!O6)/(Workings!L6+Workings!N6),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I7" s="11"/>
-      <c r="J7" s="12" t="s">
-        <v>15</v>
+      <c r="J7" s="11"/>
+      <c r="K7" s="12" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">(Workings!B7*Workings!C7+Workings!D7*Workings!E7+Workings!F7*Workings!G7+Workings!H7*Workings!I7+Workings!J7*Workings!K7+Workings!L7*Workings!M7+Workings!N7*Workings!O7)*1000/10000000</f>
@@ -1178,15 +1197,19 @@
         <f aca="false">B8*10000000/(F8*1000000)</f>
         <v>3.84196851361721</v>
       </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L7*Workings!M7+Workings!N7*Workings!O7)/(Workings!L7+Workings!N7),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I8" s="11"/>
-      <c r="J8" s="12" t="s">
-        <v>15</v>
+      <c r="J8" s="11"/>
+      <c r="K8" s="12" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">(Workings!B8*Workings!C8+Workings!D8*Workings!E8+Workings!F8*Workings!G8+Workings!H8*Workings!I8+Workings!J8*Workings!K8+Workings!L8*Workings!M8+Workings!N8*Workings!O8)*1000/10000000</f>
@@ -1212,15 +1235,19 @@
         <f aca="false">B9*10000000/(F9*1000000)</f>
         <v>4.17952328276617</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L8*Workings!M8+Workings!N8*Workings!O8)/(Workings!L8+Workings!N8),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I9" s="11"/>
-      <c r="J9" s="12" t="s">
-        <v>18</v>
+      <c r="J9" s="11"/>
+      <c r="K9" s="12" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">(Workings!B9*Workings!C9+Workings!D9*Workings!E9+Workings!F9*Workings!G9+Workings!H9*Workings!I9+Workings!J9*Workings!K9+Workings!L9*Workings!M9+Workings!N9*Workings!O9)*1000/10000000</f>
@@ -1246,15 +1273,19 @@
         <f aca="false">B10*10000000/(F10*1000000)</f>
         <v>4.13615162495439</v>
       </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L9*Workings!M9+Workings!N9*Workings!O9)/(Workings!L9+Workings!N9),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I10" s="11"/>
-      <c r="J10" s="12" t="s">
-        <v>18</v>
+      <c r="J10" s="11"/>
+      <c r="K10" s="12" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">(Workings!B10*Workings!C10+Workings!D10*Workings!E10+Workings!F10*Workings!G10+Workings!H10*Workings!I10+Workings!J10*Workings!K10+Workings!L10*Workings!M10+Workings!N10*Workings!O10)*1000/10000000</f>
@@ -1280,15 +1311,19 @@
         <f aca="false">B11*10000000/(F11*1000000)</f>
         <v>4.42124768562647</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L10*Workings!M10+Workings!N10*Workings!O10)/(Workings!L10+Workings!N10),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I11" s="11"/>
-      <c r="J11" s="12" t="s">
-        <v>21</v>
+      <c r="J11" s="11"/>
+      <c r="K11" s="12" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">(Workings!B11*Workings!C11+Workings!D11*Workings!E11+Workings!F11*Workings!G11+Workings!H11*Workings!I11+Workings!J11*Workings!K11+Workings!L11*Workings!M11+Workings!N11*Workings!O11)*1000/10000000</f>
@@ -1314,15 +1349,19 @@
         <f aca="false">B12*10000000/(F12*1000000)</f>
         <v>3.70170330580701</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L11*Workings!M11+Workings!N11*Workings!O11)/(Workings!L11+Workings!N11),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I12" s="11"/>
-      <c r="J12" s="12" t="s">
-        <v>21</v>
+      <c r="J12" s="11"/>
+      <c r="K12" s="12" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" s="7" t="n">
         <f aca="false">(Workings!B12*Workings!C12+Workings!D12*Workings!E12+Workings!F12*Workings!G12+Workings!H12*Workings!I12+Workings!J12*Workings!K12+Workings!L12*Workings!M12+Workings!N12*Workings!O12)*1000/10000000</f>
@@ -1348,15 +1387,19 @@
         <f aca="false">B13*10000000/(F13*1000000)</f>
         <v>4.13400682555015</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L12*Workings!M12+Workings!N12*Workings!O12)/(Workings!L12+Workings!N12),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I13" s="11"/>
-      <c r="J13" s="12" t="s">
-        <v>24</v>
+      <c r="J13" s="11"/>
+      <c r="K13" s="12" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">(Workings!B13*Workings!C13+Workings!D13*Workings!E13+Workings!F13*Workings!G13+Workings!H13*Workings!I13+Workings!J13*Workings!K13+Workings!L13*Workings!M13+Workings!N13*Workings!O13)*1000/10000000</f>
@@ -1382,15 +1425,19 @@
         <f aca="false">B14*10000000/(F14*1000000)</f>
         <v>4.62030805368421</v>
       </c>
-      <c r="H14" s="11"/>
+      <c r="H14" s="10" t="str">
+        <f aca="false">IFERROR((Workings!L13*Workings!M13+Workings!N13*Workings!O13)/(Workings!L13+Workings!N13),"-")</f>
+        <v>-</v>
+      </c>
       <c r="I14" s="11"/>
-      <c r="J14" s="12" t="s">
-        <v>24</v>
+      <c r="J14" s="11"/>
+      <c r="K14" s="12" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">(Workings!B14*Workings!C14+Workings!D14*Workings!E14+Workings!F14*Workings!G14+Workings!H14*Workings!I14+Workings!J14*Workings!K14+Workings!L14*Workings!M14+Workings!N14*Workings!O14)*1000/10000000</f>
@@ -1416,15 +1463,19 @@
         <f aca="false">B15*10000000/(F15*1000000)</f>
         <v>4.71773889826559</v>
       </c>
-      <c r="H15" s="11"/>
+      <c r="H15" s="10" t="n">
+        <f aca="false">IFERROR((Workings!L14*Workings!M14+Workings!N14*Workings!O14)/(Workings!L14+Workings!N14),"-")</f>
+        <v>0.577239530132789</v>
+      </c>
       <c r="I15" s="11"/>
-      <c r="J15" s="12" t="s">
-        <v>27</v>
+      <c r="J15" s="11"/>
+      <c r="K15" s="12" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">(Workings!B15*Workings!C15+Workings!D15*Workings!E15+Workings!F15*Workings!G15+Workings!H15*Workings!I15+Workings!J15*Workings!K15+Workings!L15*Workings!M15+Workings!N15*Workings!O15)*1000/10000000</f>
@@ -1450,15 +1501,19 @@
         <f aca="false">B16*10000000/(F16*1000000)</f>
         <v>4.57637623302898</v>
       </c>
-      <c r="H16" s="11"/>
+      <c r="H16" s="10" t="n">
+        <f aca="false">IFERROR((Workings!L15*Workings!M15+Workings!N15*Workings!O15)/(Workings!L15+Workings!N15),"-")</f>
+        <v>1.12141795541273</v>
+      </c>
       <c r="I16" s="11"/>
-      <c r="J16" s="12" t="s">
-        <v>27</v>
+      <c r="J16" s="11"/>
+      <c r="K16" s="12" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1469,298 +1524,326 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K19" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J19" s="12" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J23" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K23" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J25" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>32</v>
+        <v>32</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1771,10 +1854,11 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B28" s="7" t="n">
         <f aca="false">SUMPRODUCT(Workings!B19:E19,Workings!F19:I19)/10</f>
@@ -1793,28 +1877,31 @@
         <v>0.0777086787911206</v>
       </c>
       <c r="F28" s="7" t="n">
-        <f aca="false">H28*Workings!J19</f>
+        <f aca="false">I28*Workings!J19</f>
         <v>8013.936</v>
       </c>
       <c r="G28" s="10" t="n">
         <f aca="false">B28*10000000/(F28*1000000)</f>
         <v>5.80094974554326</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I28" s="8" t="n">
         <f aca="false">SUM(Workings!B19:E19)</f>
         <v>112.24</v>
       </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">B28*10/H28</f>
+      <c r="J28" s="7" t="n">
+        <f aca="false">B28*10/I28</f>
         <v>414.187811831789</v>
       </c>
-      <c r="J28" s="12" t="s">
-        <v>43</v>
+      <c r="K28" s="12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29" s="7" t="n">
         <f aca="false">SUMPRODUCT(Workings!B20:E20,Workings!F20:I20)/10</f>
@@ -1833,28 +1920,32 @@
         <v>0.0779810947673017</v>
       </c>
       <c r="F29" s="7" t="n">
-        <f aca="false">H29*Workings!J20</f>
+        <f aca="false">I29*Workings!J20</f>
         <v>8845.277</v>
       </c>
       <c r="G29" s="10" t="n">
         <f aca="false">B29*10000000/(F29*1000000)</f>
         <v>5.48407246036501</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="10" t="n">
+        <f aca="false">'Source Rates'!H26</f>
+        <v>4.47266339470358</v>
+      </c>
+      <c r="I29" s="8" t="n">
         <f aca="false">SUM(Workings!B20:E20)</f>
         <v>125.11</v>
       </c>
-      <c r="I29" s="7" t="n">
-        <f aca="false">B29*10/H29</f>
+      <c r="J29" s="7" t="n">
+        <f aca="false">B29*10/I29</f>
         <v>387.723922947806</v>
       </c>
-      <c r="J29" s="12" t="s">
-        <v>45</v>
+      <c r="K29" s="12" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B30" s="7" t="n">
         <f aca="false">SUMPRODUCT(Workings!B21:E21,Workings!F21:I21)/10</f>
@@ -1873,34 +1964,38 @@
         <v>0.0690161463787394</v>
       </c>
       <c r="F30" s="7" t="n">
-        <f aca="false">H30*Workings!J21</f>
+        <f aca="false">I30*Workings!J21</f>
         <v>9646</v>
       </c>
       <c r="G30" s="10" t="n">
         <f aca="false">B30*10000000/(F30*1000000)</f>
         <v>5.0560802405142</v>
       </c>
-      <c r="H30" s="8" t="n">
+      <c r="H30" s="10" t="n">
+        <f aca="false">'Source Rates'!H27</f>
+        <v>4.48409759441102</v>
+      </c>
+      <c r="I30" s="8" t="n">
         <f aca="false">SUM(Workings!B21:E21)</f>
         <v>140</v>
       </c>
-      <c r="I30" s="7" t="n">
-        <f aca="false">B30*10/H30</f>
+      <c r="J30" s="7" t="n">
+        <f aca="false">B30*10/I30</f>
         <v>348.363928571429</v>
       </c>
-      <c r="J30" s="12" t="s">
-        <v>47</v>
+      <c r="K30" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B31" s="15" t="n">
         <f aca="false">B30/140*134.67</f>
         <v>4691.41702607143</v>
       </c>
-      <c r="C31" s="15" t="n">
+      <c r="C31" s="16" t="n">
         <f aca="false">B31/100</f>
         <v>46.9141702607143</v>
       </c>
@@ -1908,7 +2003,7 @@
         <f aca="false">D30</f>
         <v>70666</v>
       </c>
-      <c r="E31" s="16" t="n">
+      <c r="E31" s="17" t="n">
         <f aca="false">B31/D31</f>
         <v>0.066388603091606</v>
       </c>
@@ -1916,8 +2011,9 @@
       <c r="G31" s="11"/>
       <c r="H31" s="11"/>
       <c r="I31" s="11"/>
-      <c r="J31" s="12" t="s">
-        <v>49</v>
+      <c r="J31" s="11"/>
+      <c r="K31" s="12" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1944,662 +2040,662 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>50</v>
+      <c r="A1" s="18" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
+      <c r="A4" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="22" t="n">
+      <c r="A6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="23" t="n">
         <v>288469</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="24" t="n">
         <v>4.23</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="23" t="n">
         <v>291512</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <v>3.61</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="23" t="n">
         <v>318523</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="24" t="n">
         <v>1.32</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="23" t="n">
         <v>306873</v>
       </c>
-      <c r="I6" s="23" t="n">
+      <c r="I6" s="24" t="n">
         <v>4.63</v>
       </c>
-      <c r="J6" s="22"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="24" t="n">
+      <c r="J6" s="23"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="25" t="n">
         <v>2606.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="22" t="n">
+      <c r="A7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>423050</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="24" t="n">
         <v>4.01</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>305267</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <v>4.27</v>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="F7" s="23" t="n">
         <v>256036</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="24" t="n">
         <v>1.41</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="23" t="n">
         <v>292707</v>
       </c>
-      <c r="I7" s="23" t="n">
+      <c r="I7" s="24" t="n">
         <v>5.28</v>
       </c>
-      <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24" t="n">
+      <c r="J7" s="23"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="25" t="n">
         <v>3299.45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="22" t="n">
+      <c r="A8" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>847582</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="24" t="n">
         <v>4.79</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>188908</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="24" t="n">
         <v>4.91</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="23" t="n">
         <v>309571</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="24" t="n">
         <v>1.4</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="23" t="n">
         <v>64249</v>
       </c>
-      <c r="I8" s="23" t="n">
+      <c r="I8" s="24" t="n">
         <v>7.4</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="23" t="n">
         <v>477.05</v>
       </c>
-      <c r="K8" s="23" t="n">
+      <c r="K8" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="L8" s="22"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="24" t="n">
+      <c r="L8" s="23"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="25" t="n">
         <v>4910.52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="22" t="n">
+      <c r="A9" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="23" t="n">
         <v>923400</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="24" t="n">
         <v>4.69</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="23" t="n">
         <v>176961</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <v>5.62</v>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="F9" s="23" t="n">
         <v>316750</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="24" t="n">
         <v>1.73</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="23" t="n">
         <v>5527</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="24" t="n">
         <v>15.05</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="J9" s="23" t="n">
         <v>19064</v>
       </c>
-      <c r="K9" s="23" t="n">
+      <c r="K9" s="24" t="n">
         <v>0.35</v>
       </c>
-      <c r="L9" s="22"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="24" t="n">
+      <c r="L9" s="23"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="25" t="n">
         <v>5509.22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="22" t="n">
+      <c r="A10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="23" t="n">
         <v>817938</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="24" t="n">
         <v>4.83</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="23" t="n">
         <v>99071</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <v>6.31</v>
       </c>
-      <c r="F10" s="22" t="n">
+      <c r="F10" s="23" t="n">
         <v>593848</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="24" t="n">
         <v>3.64</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="23" t="n">
         <v>1394</v>
       </c>
-      <c r="I10" s="23" t="n">
+      <c r="I10" s="24" t="n">
         <v>19.78</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="23" t="n">
         <v>19481</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="24" t="n">
         <v>0.37</v>
       </c>
-      <c r="L10" s="22"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="24" t="n">
+      <c r="L10" s="23"/>
+      <c r="M10" s="24"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="25" t="n">
         <v>6383</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="22" t="n">
+      <c r="A11" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="23" t="n">
         <v>361072</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="24" t="n">
         <v>5.02</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="23" t="n">
         <v>61264</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="24" t="n">
         <v>6.99</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F11" s="23" t="n">
         <v>1187204</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="24" t="n">
         <v>3.17</v>
       </c>
-      <c r="H11" s="22"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="22" t="n">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="23" t="n">
         <v>13997</v>
       </c>
-      <c r="K11" s="23" t="n">
+      <c r="K11" s="24" t="n">
         <v>0.4</v>
       </c>
-      <c r="L11" s="22"/>
-      <c r="M11" s="23"/>
-      <c r="N11" s="22"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="24" t="n">
+      <c r="L11" s="23"/>
+      <c r="M11" s="24"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="25" t="n">
         <v>7050</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="22" t="n">
+      <c r="A12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="23" t="n">
         <v>543606</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="24" t="n">
         <v>5.35</v>
       </c>
-      <c r="D12" s="22" t="n">
+      <c r="D12" s="23" t="n">
         <v>71112</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="24" t="n">
         <v>9.07</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="23" t="n">
         <v>2251369</v>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G12" s="24" t="n">
         <v>3.71</v>
       </c>
-      <c r="H12" s="22"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="22" t="n">
+      <c r="H12" s="23"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="23" t="n">
         <v>16025</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="K12" s="24" t="n">
         <v>0.55</v>
       </c>
-      <c r="L12" s="22"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="22"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="24" t="n">
+      <c r="L12" s="23"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="25" t="n">
         <v>13206</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="22" t="n">
+      <c r="A13" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="23" t="n">
         <v>663933</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="24" t="n">
         <v>5.54</v>
       </c>
-      <c r="D13" s="22" t="n">
+      <c r="D13" s="23" t="n">
         <v>55640</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="24" t="n">
         <v>13.8</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="23" t="n">
         <v>2588989</v>
       </c>
-      <c r="G13" s="23" t="n">
+      <c r="G13" s="24" t="n">
         <v>4.21</v>
       </c>
-      <c r="H13" s="22"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="22" t="n">
+      <c r="H13" s="23"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="23" t="n">
         <v>14203</v>
       </c>
-      <c r="K13" s="23" t="n">
+      <c r="K13" s="24" t="n">
         <v>0.46</v>
       </c>
-      <c r="L13" s="22"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="22"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="24" t="n">
+      <c r="L13" s="23"/>
+      <c r="M13" s="24"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="25" t="n">
         <v>18158</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="22" t="n">
+      <c r="A14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="23" t="n">
         <v>652499</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="24" t="n">
         <v>6.33</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="23" t="n">
         <v>62995</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="24" t="n">
         <v>13.57</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="23" t="n">
         <v>2719775</v>
       </c>
-      <c r="G14" s="23" t="n">
+      <c r="G14" s="24" t="n">
         <v>4.15</v>
       </c>
-      <c r="H14" s="22"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="22" t="n">
+      <c r="H14" s="23"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="23" t="n">
         <v>11447</v>
       </c>
-      <c r="K14" s="23" t="n">
+      <c r="K14" s="24" t="n">
         <v>0.41</v>
       </c>
-      <c r="L14" s="22" t="n">
+      <c r="L14" s="23" t="n">
         <v>2065</v>
       </c>
-      <c r="M14" s="23" t="n">
+      <c r="M14" s="24" t="n">
         <v>0.27</v>
       </c>
-      <c r="N14" s="22" t="n">
+      <c r="N14" s="23" t="n">
         <v>1851</v>
       </c>
-      <c r="O14" s="23" t="n">
+      <c r="O14" s="24" t="n">
         <v>0.92</v>
       </c>
-      <c r="P14" s="24" t="n">
+      <c r="P14" s="25" t="n">
         <v>20023</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="22" t="n">
+      <c r="A15" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="23" t="n">
         <v>583398</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="24" t="n">
         <v>6.67</v>
       </c>
-      <c r="D15" s="22" t="n">
+      <c r="D15" s="23" t="n">
         <v>35818</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="24" t="n">
         <v>14.76</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="23" t="n">
         <v>2735008</v>
       </c>
-      <c r="G15" s="23" t="n">
+      <c r="G15" s="24" t="n">
         <v>4.02</v>
       </c>
-      <c r="H15" s="22"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="22" t="n">
+      <c r="H15" s="23"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="23" t="n">
         <v>10953</v>
       </c>
-      <c r="K15" s="23" t="n">
+      <c r="K15" s="24" t="n">
         <v>0.26</v>
       </c>
-      <c r="L15" s="22" t="n">
+      <c r="L15" s="23" t="n">
         <v>2928</v>
       </c>
-      <c r="M15" s="23" t="n">
+      <c r="M15" s="24" t="n">
         <v>0.52</v>
       </c>
-      <c r="N15" s="22" t="n">
+      <c r="N15" s="23" t="n">
         <v>2051</v>
       </c>
-      <c r="O15" s="23" t="n">
+      <c r="O15" s="24" t="n">
         <v>1.98</v>
       </c>
-      <c r="P15" s="24" t="n">
+      <c r="P15" s="25" t="n">
         <v>20078</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
-      <c r="O17" s="19"/>
-      <c r="P17" s="19"/>
+      <c r="A17" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="20"/>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="23" t="n">
+      <c r="A19" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="24" t="n">
         <v>28.5</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="24" t="n">
         <v>25.08</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="24" t="n">
         <v>25.44</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="24" t="n">
         <v>33.22</v>
       </c>
-      <c r="F19" s="24" t="n">
+      <c r="F19" s="25" t="n">
         <v>413</v>
       </c>
-      <c r="G19" s="24" t="n">
+      <c r="G19" s="25" t="n">
         <v>431</v>
       </c>
-      <c r="H19" s="24" t="n">
+      <c r="H19" s="25" t="n">
         <v>424</v>
       </c>
-      <c r="I19" s="24" t="n">
+      <c r="I19" s="25" t="n">
         <v>395</v>
       </c>
-      <c r="J19" s="25" t="n">
+      <c r="J19" s="26" t="n">
         <v>71.4</v>
       </c>
-      <c r="K19" s="24" t="n">
+      <c r="K19" s="25" t="n">
         <v>59824</v>
       </c>
-      <c r="L19" s="24" t="n">
+      <c r="L19" s="25" t="n">
         <v>69810</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="23" t="n">
+      <c r="A20" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="24" t="n">
         <v>31.91</v>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="24" t="n">
         <v>27.28</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="24" t="n">
         <v>29.45</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="24" t="n">
         <v>36.47</v>
       </c>
-      <c r="F20" s="24" t="n">
+      <c r="F20" s="25" t="n">
         <v>389</v>
       </c>
-      <c r="G20" s="24" t="n">
+      <c r="G20" s="25" t="n">
         <v>403</v>
       </c>
-      <c r="H20" s="24" t="n">
+      <c r="H20" s="25" t="n">
         <v>409</v>
       </c>
-      <c r="I20" s="24" t="n">
+      <c r="I20" s="25" t="n">
         <v>358</v>
       </c>
-      <c r="J20" s="25" t="n">
+      <c r="J20" s="26" t="n">
         <v>70.7</v>
       </c>
-      <c r="K20" s="24" t="n">
+      <c r="K20" s="25" t="n">
         <v>62205</v>
       </c>
-      <c r="L20" s="24" t="n">
+      <c r="L20" s="25" t="n">
         <v>74936</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="23" t="n">
+      <c r="A21" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="24" t="n">
         <v>33.07</v>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="24" t="n">
         <v>29.9</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="24" t="n">
         <v>35.02</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="24" t="n">
         <v>42.01</v>
       </c>
-      <c r="F21" s="24" t="n">
+      <c r="F21" s="25" t="n">
         <v>356</v>
       </c>
-      <c r="G21" s="24" t="n">
+      <c r="G21" s="25" t="n">
         <v>372</v>
       </c>
-      <c r="H21" s="24" t="n">
+      <c r="H21" s="25" t="n">
         <v>349</v>
       </c>
-      <c r="I21" s="24" t="n">
+      <c r="I21" s="25" t="n">
         <v>325</v>
       </c>
-      <c r="J21" s="25" t="n">
+      <c r="J21" s="26" t="n">
         <v>68.9</v>
       </c>
-      <c r="K21" s="24" t="n">
+      <c r="K21" s="25" t="n">
         <v>70666</v>
       </c>
-      <c r="L21" s="24" t="n">
+      <c r="L21" s="25" t="n">
         <v>87384</v>
       </c>
     </row>
@@ -2619,7 +2715,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -2627,796 +2723,849 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>80</v>
+      <c r="A1" s="18" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
+      <c r="A4" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I5" s="26" t="s">
         <v>90</v>
       </c>
+      <c r="I5" s="27" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="27" t="n">
+      <c r="A6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="28" t="n">
         <f aca="false">IF(Workings!C6="","",Workings!C6)</f>
         <v>4.23</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="28" t="n">
         <f aca="false">IF(Workings!E6="","",Workings!E6)</f>
         <v>3.61</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="28" t="n">
         <f aca="false">IF(Workings!G6="","",Workings!G6)</f>
         <v>1.32</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="28" t="n">
         <f aca="false">IF(Workings!I6="","",Workings!I6)</f>
         <v>4.63</v>
       </c>
-      <c r="F6" s="27" t="str">
+      <c r="F6" s="28" t="str">
         <f aca="false">IF(Workings!K6="","",Workings!K6)</f>
         <v/>
       </c>
-      <c r="G6" s="27" t="str">
+      <c r="G6" s="28" t="str">
         <f aca="false">IF(Workings!M6="","",Workings!M6)</f>
         <v/>
       </c>
-      <c r="H6" s="27" t="str">
+      <c r="H6" s="28" t="str">
         <f aca="false">IF(Workings!O6="","",Workings!O6)</f>
         <v/>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="29" t="n">
         <f aca="false">'Time Series'!G7</f>
         <v>3.41291939368347</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="27" t="n">
+      <c r="A7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="28" t="n">
         <f aca="false">IF(Workings!C7="","",Workings!C7)</f>
         <v>4.01</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="28" t="n">
         <f aca="false">IF(Workings!E7="","",Workings!E7)</f>
         <v>4.27</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="28" t="n">
         <f aca="false">IF(Workings!G7="","",Workings!G7)</f>
         <v>1.41</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">IF(Workings!I7="","",Workings!I7)</f>
         <v>5.28</v>
       </c>
-      <c r="F7" s="27" t="str">
+      <c r="F7" s="28" t="str">
         <f aca="false">IF(Workings!K7="","",Workings!K7)</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="str">
+      <c r="G7" s="28" t="str">
         <f aca="false">IF(Workings!M7="","",Workings!M7)</f>
         <v/>
       </c>
-      <c r="H7" s="27" t="str">
+      <c r="H7" s="28" t="str">
         <f aca="false">IF(Workings!O7="","",Workings!O7)</f>
         <v/>
       </c>
-      <c r="I7" s="28" t="n">
+      <c r="I7" s="29" t="n">
         <f aca="false">'Time Series'!G8</f>
         <v>3.84196851361721</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="27" t="n">
+      <c r="A8" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="28" t="n">
         <f aca="false">IF(Workings!C8="","",Workings!C8)</f>
         <v>4.79</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="28" t="n">
         <f aca="false">IF(Workings!E8="","",Workings!E8)</f>
         <v>4.91</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="28" t="n">
         <f aca="false">IF(Workings!G8="","",Workings!G8)</f>
         <v>1.4</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="28" t="n">
         <f aca="false">IF(Workings!I8="","",Workings!I8)</f>
         <v>7.4</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="28" t="n">
         <f aca="false">IF(Workings!K8="","",Workings!K8)</f>
         <v>0.25</v>
       </c>
-      <c r="G8" s="27" t="str">
+      <c r="G8" s="28" t="str">
         <f aca="false">IF(Workings!M8="","",Workings!M8)</f>
         <v/>
       </c>
-      <c r="H8" s="27" t="str">
+      <c r="H8" s="28" t="str">
         <f aca="false">IF(Workings!O8="","",Workings!O8)</f>
         <v/>
       </c>
-      <c r="I8" s="28" t="n">
+      <c r="I8" s="29" t="n">
         <f aca="false">'Time Series'!G9</f>
         <v>4.17952328276617</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="27" t="n">
+      <c r="A9" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="28" t="n">
         <f aca="false">IF(Workings!C9="","",Workings!C9)</f>
         <v>4.69</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="28" t="n">
         <f aca="false">IF(Workings!E9="","",Workings!E9)</f>
         <v>5.62</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="28" t="n">
         <f aca="false">IF(Workings!G9="","",Workings!G9)</f>
         <v>1.73</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="28" t="n">
         <f aca="false">IF(Workings!I9="","",Workings!I9)</f>
         <v>15.05</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="28" t="n">
         <f aca="false">IF(Workings!K9="","",Workings!K9)</f>
         <v>0.35</v>
       </c>
-      <c r="G9" s="27" t="str">
+      <c r="G9" s="28" t="str">
         <f aca="false">IF(Workings!M9="","",Workings!M9)</f>
         <v/>
       </c>
-      <c r="H9" s="27" t="str">
+      <c r="H9" s="28" t="str">
         <f aca="false">IF(Workings!O9="","",Workings!O9)</f>
         <v/>
       </c>
-      <c r="I9" s="28" t="n">
+      <c r="I9" s="29" t="n">
         <f aca="false">'Time Series'!G10</f>
         <v>4.13615162495439</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="27" t="n">
+      <c r="A10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="28" t="n">
         <f aca="false">IF(Workings!C10="","",Workings!C10)</f>
         <v>4.83</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="28" t="n">
         <f aca="false">IF(Workings!E10="","",Workings!E10)</f>
         <v>6.31</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="28" t="n">
         <f aca="false">IF(Workings!G10="","",Workings!G10)</f>
         <v>3.64</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">IF(Workings!I10="","",Workings!I10)</f>
         <v>19.78</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="28" t="n">
         <f aca="false">IF(Workings!K10="","",Workings!K10)</f>
         <v>0.37</v>
       </c>
-      <c r="G10" s="27" t="str">
+      <c r="G10" s="28" t="str">
         <f aca="false">IF(Workings!M10="","",Workings!M10)</f>
         <v/>
       </c>
-      <c r="H10" s="27" t="str">
+      <c r="H10" s="28" t="str">
         <f aca="false">IF(Workings!O10="","",Workings!O10)</f>
         <v/>
       </c>
-      <c r="I10" s="28" t="n">
+      <c r="I10" s="29" t="n">
         <f aca="false">'Time Series'!G11</f>
         <v>4.42124768562647</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="27" t="n">
+      <c r="A11" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="28" t="n">
         <f aca="false">IF(Workings!C11="","",Workings!C11)</f>
         <v>5.02</v>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="28" t="n">
         <f aca="false">IF(Workings!E11="","",Workings!E11)</f>
         <v>6.99</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="28" t="n">
         <f aca="false">IF(Workings!G11="","",Workings!G11)</f>
         <v>3.17</v>
       </c>
-      <c r="E11" s="27" t="str">
+      <c r="E11" s="28" t="str">
         <f aca="false">IF(Workings!I11="","",Workings!I11)</f>
         <v/>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="28" t="n">
         <f aca="false">IF(Workings!K11="","",Workings!K11)</f>
         <v>0.4</v>
       </c>
-      <c r="G11" s="27" t="str">
+      <c r="G11" s="28" t="str">
         <f aca="false">IF(Workings!M11="","",Workings!M11)</f>
         <v/>
       </c>
-      <c r="H11" s="27" t="str">
+      <c r="H11" s="28" t="str">
         <f aca="false">IF(Workings!O11="","",Workings!O11)</f>
         <v/>
       </c>
-      <c r="I11" s="28" t="n">
+      <c r="I11" s="29" t="n">
         <f aca="false">'Time Series'!G12</f>
         <v>3.70170330580701</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="27" t="n">
+      <c r="A12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="28" t="n">
         <f aca="false">IF(Workings!C12="","",Workings!C12)</f>
         <v>5.35</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="28" t="n">
         <f aca="false">IF(Workings!E12="","",Workings!E12)</f>
         <v>9.07</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="28" t="n">
         <f aca="false">IF(Workings!G12="","",Workings!G12)</f>
         <v>3.71</v>
       </c>
-      <c r="E12" s="27" t="str">
+      <c r="E12" s="28" t="str">
         <f aca="false">IF(Workings!I12="","",Workings!I12)</f>
         <v/>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <f aca="false">IF(Workings!K12="","",Workings!K12)</f>
         <v>0.55</v>
       </c>
-      <c r="G12" s="27" t="str">
+      <c r="G12" s="28" t="str">
         <f aca="false">IF(Workings!M12="","",Workings!M12)</f>
         <v/>
       </c>
-      <c r="H12" s="27" t="str">
+      <c r="H12" s="28" t="str">
         <f aca="false">IF(Workings!O12="","",Workings!O12)</f>
         <v/>
       </c>
-      <c r="I12" s="28" t="n">
+      <c r="I12" s="29" t="n">
         <f aca="false">'Time Series'!G13</f>
         <v>4.13400682555015</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="27" t="n">
+      <c r="A13" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="28" t="n">
         <f aca="false">IF(Workings!C13="","",Workings!C13)</f>
         <v>5.54</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="28" t="n">
         <f aca="false">IF(Workings!E13="","",Workings!E13)</f>
         <v>13.8</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="28" t="n">
         <f aca="false">IF(Workings!G13="","",Workings!G13)</f>
         <v>4.21</v>
       </c>
-      <c r="E13" s="27" t="str">
+      <c r="E13" s="28" t="str">
         <f aca="false">IF(Workings!I13="","",Workings!I13)</f>
         <v/>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="28" t="n">
         <f aca="false">IF(Workings!K13="","",Workings!K13)</f>
         <v>0.46</v>
       </c>
-      <c r="G13" s="27" t="str">
+      <c r="G13" s="28" t="str">
         <f aca="false">IF(Workings!M13="","",Workings!M13)</f>
         <v/>
       </c>
-      <c r="H13" s="27" t="str">
+      <c r="H13" s="28" t="str">
         <f aca="false">IF(Workings!O13="","",Workings!O13)</f>
         <v/>
       </c>
-      <c r="I13" s="28" t="n">
+      <c r="I13" s="29" t="n">
         <f aca="false">'Time Series'!G14</f>
         <v>4.62030805368421</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="27" t="n">
+      <c r="A14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="28" t="n">
         <f aca="false">IF(Workings!C14="","",Workings!C14)</f>
         <v>6.33</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="28" t="n">
         <f aca="false">IF(Workings!E14="","",Workings!E14)</f>
         <v>13.57</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="28" t="n">
         <f aca="false">IF(Workings!G14="","",Workings!G14)</f>
         <v>4.15</v>
       </c>
-      <c r="E14" s="27" t="str">
+      <c r="E14" s="28" t="str">
         <f aca="false">IF(Workings!I14="","",Workings!I14)</f>
         <v/>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="28" t="n">
         <f aca="false">IF(Workings!K14="","",Workings!K14)</f>
         <v>0.41</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="28" t="n">
         <f aca="false">IF(Workings!M14="","",Workings!M14)</f>
         <v>0.27</v>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="28" t="n">
         <f aca="false">IF(Workings!O14="","",Workings!O14)</f>
         <v>0.92</v>
       </c>
-      <c r="I14" s="28" t="n">
+      <c r="I14" s="29" t="n">
         <f aca="false">'Time Series'!G15</f>
         <v>4.71773889826559</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="27" t="n">
+      <c r="A15" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="28" t="n">
         <f aca="false">IF(Workings!C15="","",Workings!C15)</f>
         <v>6.67</v>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="28" t="n">
         <f aca="false">IF(Workings!E15="","",Workings!E15)</f>
         <v>14.76</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="28" t="n">
         <f aca="false">IF(Workings!G15="","",Workings!G15)</f>
         <v>4.02</v>
       </c>
-      <c r="E15" s="27" t="str">
+      <c r="E15" s="28" t="str">
         <f aca="false">IF(Workings!I15="","",Workings!I15)</f>
         <v/>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="28" t="n">
         <f aca="false">IF(Workings!K15="","",Workings!K15)</f>
         <v>0.26</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="28" t="n">
         <f aca="false">IF(Workings!M15="","",Workings!M15)</f>
         <v>0.52</v>
       </c>
-      <c r="H15" s="27" t="n">
+      <c r="H15" s="28" t="n">
         <f aca="false">IF(Workings!O15="","",Workings!O15)</f>
         <v>1.98</v>
       </c>
-      <c r="I15" s="28" t="n">
+      <c r="I15" s="29" t="n">
         <f aca="false">'Time Series'!G16</f>
         <v>4.57637623302898</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
+      <c r="A17" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
-        <v>92</v>
+      <c r="A18" s="21" t="s">
+        <v>93</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="K18" s="26" t="s">
         <v>102</v>
       </c>
+      <c r="K18" s="27" t="s">
+        <v>103</v>
+      </c>
       <c r="L18" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="B19" s="29" t="n">
+      <c r="A19" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="30" t="n">
         <v>0.461</v>
       </c>
-      <c r="C19" s="29" t="n">
+      <c r="C19" s="30" t="n">
         <v>0.237</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="30" t="n">
         <v>0.128</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="30" t="n">
         <v>0.174</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="24" t="n">
         <v>7.1</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="24" t="n">
         <v>6.7</v>
       </c>
-      <c r="H19" s="23" t="n">
+      <c r="H19" s="24" t="n">
         <v>4.6</v>
       </c>
-      <c r="I19" s="23" t="n">
+      <c r="I19" s="24" t="n">
         <v>0.7</v>
       </c>
-      <c r="J19" s="30" t="n">
+      <c r="J19" s="31" t="n">
         <v>5.6</v>
       </c>
-      <c r="K19" s="23" t="n">
+      <c r="K19" s="24" t="n">
         <v>72.4</v>
       </c>
+      <c r="L19" s="32" t="n">
+        <f aca="false">Workings!C20*K19</f>
+        <v>1975.072</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="29" t="n">
+      <c r="A20" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="30" t="n">
         <v>0.454</v>
       </c>
-      <c r="C20" s="29" t="n">
+      <c r="C20" s="30" t="n">
         <v>0.231</v>
       </c>
-      <c r="D20" s="29" t="n">
+      <c r="D20" s="30" t="n">
         <v>0.127</v>
       </c>
-      <c r="E20" s="29" t="n">
+      <c r="E20" s="30" t="n">
         <v>0.187</v>
       </c>
-      <c r="F20" s="23" t="n">
+      <c r="F20" s="24" t="n">
         <v>7.1</v>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="24" t="n">
         <v>8.1</v>
       </c>
-      <c r="H20" s="23" t="n">
+      <c r="H20" s="24" t="n">
         <v>4.5</v>
       </c>
-      <c r="I20" s="23" t="n">
+      <c r="I20" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="J20" s="30" t="n">
+      <c r="J20" s="31" t="n">
         <v>5.8</v>
       </c>
-      <c r="K20" s="23" t="n">
+      <c r="K20" s="24" t="n">
         <v>70.8</v>
       </c>
+      <c r="L20" s="32" t="n">
+        <f aca="false">Workings!D20*K20</f>
+        <v>2085.06</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="29" t="n">
+      <c r="A21" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="30" t="n">
         <v>0.42</v>
       </c>
-      <c r="C21" s="29" t="n">
+      <c r="C21" s="30" t="n">
         <v>0.236</v>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="30" t="n">
         <v>0.139</v>
       </c>
-      <c r="E21" s="29" t="n">
+      <c r="E21" s="30" t="n">
         <v>0.205</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="24" t="n">
         <v>6.48</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="24" t="n">
         <v>6.97</v>
       </c>
-      <c r="H21" s="23" t="n">
+      <c r="H21" s="24" t="n">
         <v>4.36</v>
       </c>
-      <c r="I21" s="23" t="n">
+      <c r="I21" s="24" t="n">
         <v>0.71</v>
       </c>
-      <c r="J21" s="30" t="n">
+      <c r="J21" s="31" t="n">
         <v>5.19</v>
       </c>
-      <c r="K21" s="23" t="n">
+      <c r="K21" s="24" t="n">
         <v>69.04</v>
       </c>
+      <c r="L21" s="32" t="n">
+        <f aca="false">Workings!E20*K21</f>
+        <v>2517.8888</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="B22" s="29" t="n">
+      <c r="A22" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="30" t="n">
         <v>0.384</v>
       </c>
-      <c r="C22" s="29" t="n">
+      <c r="C22" s="30" t="n">
         <v>0.221</v>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="30" t="n">
         <v>0.191</v>
       </c>
-      <c r="E22" s="29" t="n">
+      <c r="E22" s="30" t="n">
         <v>0.204</v>
       </c>
-      <c r="F22" s="23" t="n">
+      <c r="F22" s="24" t="n">
         <v>6.7</v>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="24" t="n">
         <v>7.1</v>
       </c>
-      <c r="H22" s="23" t="n">
+      <c r="H22" s="24" t="n">
         <v>4.5</v>
       </c>
-      <c r="I22" s="23" t="n">
+      <c r="I22" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="J22" s="30" t="n">
+      <c r="J22" s="31" t="n">
         <v>5.1</v>
       </c>
-      <c r="K22" s="23" t="n">
+      <c r="K22" s="24" t="n">
         <v>69.3</v>
       </c>
-      <c r="L22" s="31" t="n">
+      <c r="L22" s="32" t="n">
         <f aca="false">Workings!B21*K22</f>
         <v>2291.751</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" s="29" t="n">
+      <c r="A23" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="30" t="n">
         <v>0.381</v>
       </c>
-      <c r="C23" s="29" t="n">
+      <c r="C23" s="30" t="n">
         <v>0.203</v>
       </c>
-      <c r="D23" s="29" t="n">
+      <c r="D23" s="30" t="n">
         <v>0.223</v>
       </c>
-      <c r="E23" s="29" t="n">
+      <c r="E23" s="30" t="n">
         <v>0.192</v>
       </c>
-      <c r="F23" s="23" t="n">
+      <c r="F23" s="24" t="n">
         <v>6.9</v>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="24" t="n">
         <v>7.1</v>
       </c>
-      <c r="H23" s="23" t="n">
+      <c r="H23" s="24" t="n">
         <v>4.6</v>
       </c>
-      <c r="I23" s="23" t="n">
+      <c r="I23" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="J23" s="30" t="n">
+      <c r="J23" s="31" t="n">
         <v>5.3</v>
       </c>
-      <c r="K23" s="23" t="n">
+      <c r="K23" s="24" t="n">
         <v>70.7</v>
       </c>
-      <c r="L23" s="31" t="n">
+      <c r="L23" s="32" t="n">
         <f aca="false">Workings!C21*K23</f>
         <v>2113.93</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="29" t="n">
+      <c r="A24" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="30" t="n">
         <v>0.358</v>
       </c>
-      <c r="C24" s="29" t="n">
+      <c r="C24" s="30" t="n">
         <v>0.22</v>
       </c>
-      <c r="D24" s="29" t="n">
+      <c r="D24" s="30" t="n">
         <v>0.206</v>
       </c>
-      <c r="E24" s="29" t="n">
+      <c r="E24" s="30" t="n">
         <v>0.215</v>
       </c>
-      <c r="F24" s="23" t="n">
+      <c r="F24" s="24" t="n">
         <v>6.5</v>
       </c>
-      <c r="G24" s="23" t="n">
+      <c r="G24" s="24" t="n">
         <v>7.4</v>
       </c>
-      <c r="H24" s="23" t="n">
+      <c r="H24" s="24" t="n">
         <v>4.4</v>
       </c>
-      <c r="I24" s="23" t="n">
+      <c r="I24" s="24" t="n">
         <v>0.7</v>
       </c>
-      <c r="J24" s="30" t="n">
+      <c r="J24" s="31" t="n">
         <v>5.1</v>
       </c>
-      <c r="K24" s="23" t="n">
+      <c r="K24" s="24" t="n">
         <v>69</v>
       </c>
-      <c r="L24" s="31" t="n">
+      <c r="L24" s="32" t="n">
         <f aca="false">Workings!D21*K24</f>
         <v>2416.38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B25" s="29" t="n">
+      <c r="A25" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="30" t="n">
         <v>0.364</v>
       </c>
-      <c r="C25" s="29" t="n">
+      <c r="C25" s="30" t="n">
         <v>0.206</v>
       </c>
-      <c r="D25" s="29" t="n">
+      <c r="D25" s="30" t="n">
         <v>0.204</v>
       </c>
-      <c r="E25" s="29" t="n">
+      <c r="E25" s="30" t="n">
         <v>0.226</v>
       </c>
-      <c r="F25" s="23" t="n">
+      <c r="F25" s="24" t="n">
         <v>5.99</v>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G25" s="24" t="n">
         <v>7.62</v>
       </c>
-      <c r="H25" s="23" t="n">
+      <c r="H25" s="24" t="n">
         <v>4.45</v>
       </c>
-      <c r="I25" s="23" t="n">
+      <c r="I25" s="24" t="n">
         <v>0.6</v>
       </c>
-      <c r="J25" s="30" t="n">
+      <c r="J25" s="31" t="n">
         <v>4.81</v>
       </c>
-      <c r="K25" s="23" t="n">
+      <c r="K25" s="24" t="n">
         <v>67.54</v>
       </c>
-      <c r="L25" s="31" t="n">
+      <c r="L25" s="32" t="n">
         <f aca="false">Workings!E21*K25</f>
         <v>2837.3554</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="s">
-        <v>111</v>
-      </c>
-      <c r="B26" s="33" t="n">
+      <c r="A26" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="B26" s="34" t="n">
+        <f aca="false">(B19*L19+B20*L20+B21*L21)/(L19+L20+L21)</f>
+        <v>0.443087490389207</v>
+      </c>
+      <c r="C26" s="34" t="n">
+        <f aca="false">(C19*L19+C20*L20+C21*L21)/(L19+L20+L21)</f>
+        <v>0.234715384420797</v>
+      </c>
+      <c r="D26" s="34" t="n">
+        <f aca="false">(D19*L19+D20*L20+D21*L21)/(L19+L20+L21)</f>
+        <v>0.131893529312039</v>
+      </c>
+      <c r="E26" s="34" t="n">
+        <f aca="false">(E19*L19+E20*L20+E21*L21)/(L19+L20+L21)</f>
+        <v>0.18998662211588</v>
+      </c>
+      <c r="F26" s="35" t="n">
+        <f aca="false">(B19*L19*F19+B20*L20*F20+B21*L21*F21)/(B19*L19+B20*L20+B21*L21)</f>
+        <v>6.87504647926987</v>
+      </c>
+      <c r="G26" s="35" t="n">
+        <f aca="false">(C19*L19*G19+C20*L20*G20+C21*L21*G21)/(C19*L19+C20*L20+C21*L21)</f>
+        <v>7.24065314448111</v>
+      </c>
+      <c r="H26" s="35" t="n">
+        <f aca="false">(D19*L19*H19+D20*L20*H20+D21*L21*H21)/(D19*L19+D20*L20+D21*L21)</f>
+        <v>4.47266339470358</v>
+      </c>
+      <c r="I26" s="35" t="n">
+        <f aca="false">(E19*L19*I19+E20*L20*I20+E21*L21*I21)/(E19*L19+E20*L20+E21*L21)</f>
+        <v>0.735329298136412</v>
+      </c>
+      <c r="J26" s="35" t="n">
+        <f aca="false">SUMPRODUCT(J19:J21,L19:L21)/SUM(L19:L21)</f>
+        <v>5.50645781965299</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="34" t="n">
         <f aca="false">(B22*L22+B23*L23+B24*L24+B25*L25)/(L22+L23+L24+L25)</f>
         <v>0.370964556368022</v>
       </c>
-      <c r="C26" s="33" t="n">
+      <c r="C27" s="34" t="n">
         <f aca="false">(C22*L22+C23*L23+C24*L24+C25*L25)/(L22+L23+L24+L25)</f>
         <v>0.212404506487576</v>
       </c>
-      <c r="D26" s="33" t="n">
+      <c r="D27" s="34" t="n">
         <f aca="false">(D22*L22+D23*L23+D24*L24+D25*L25)/(L22+L23+L24+L25)</f>
         <v>0.20557407718752</v>
       </c>
-      <c r="E26" s="33" t="n">
+      <c r="E27" s="34" t="n">
         <f aca="false">(E22*L22+E23*L23+E24*L24+E25*L25)/(L22+L23+L24+L25)</f>
         <v>0.210587855431929</v>
       </c>
-      <c r="F26" s="34" t="n">
+      <c r="F27" s="35" t="n">
         <f aca="false">(B22*L22*F22+B23*L23*F23+B24*L24*F24+B25*L25*F25)/(B22*L22+B23*L23+B24*L24+B25*L25)</f>
         <v>6.4920304638927</v>
       </c>
-      <c r="G26" s="34" t="n">
+      <c r="G27" s="35" t="n">
         <f aca="false">(C22*L22*G22+C23*L23*G23+C24*L24*G24+C25*L25*G25)/(C22*L22+C23*L23+C24*L24+C25*L25)</f>
         <v>7.32587014832754</v>
       </c>
-      <c r="H26" s="34" t="n">
+      <c r="H27" s="35" t="n">
         <f aca="false">(D22*L22*H22+D23*L23*H23+D24*L24*H24+D25*L25*H25)/(D22*L22+D23*L23+D24*L24+D25*L25)</f>
         <v>4.48409759441102</v>
       </c>
-      <c r="I26" s="34" t="n">
+      <c r="I27" s="35" t="n">
         <f aca="false">(E22*L22*I22+E23*L23*I23+E24*L24*I24+E25*L25*I25)/(E22*L22+E23*L23+E24*L24+E25*L25)</f>
         <v>0.711412569547542</v>
       </c>
-      <c r="J26" s="34" t="n">
+      <c r="J27" s="35" t="n">
         <f aca="false">'Time Series'!G30</f>
         <v>5.0560802405142</v>
       </c>
-      <c r="K26" s="34" t="n">
+      <c r="K27" s="35" t="n">
         <f aca="false">Workings!J21</f>
         <v>68.9</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="J27" s="34" t="n">
-        <f aca="false">((B26*F26)+(C26*G26)+(D26*H26))/(B26+C26+D26)</f>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="J28" s="35" t="n">
+        <f aca="false">((B27*F27)+(C27*G27)+(D27*H27))/(B27+C27+D27)</f>
         <v>6.19331737789873</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>113</v>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -3443,178 +3592,178 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="35" t="s">
-        <v>114</v>
+      <c r="B1" s="36" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="36"/>
+      <c r="B2" s="37"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="37" t="s">
-        <v>115</v>
+      <c r="B3" s="38" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="36" t="s">
-        <v>116</v>
+      <c r="B4" s="37" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="36"/>
+      <c r="B5" s="37"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="37" t="s">
-        <v>117</v>
+      <c r="B6" s="38" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="36" t="s">
-        <v>118</v>
+      <c r="B7" s="37" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="36" t="s">
-        <v>119</v>
+      <c r="B8" s="37" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="36" t="s">
-        <v>120</v>
+      <c r="B9" s="37" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="36"/>
+      <c r="B10" s="37"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="37" t="s">
-        <v>121</v>
+      <c r="B11" s="38" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="36" t="s">
-        <v>122</v>
+      <c r="B12" s="37" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="36" t="s">
-        <v>123</v>
+      <c r="B13" s="37" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="36"/>
+      <c r="B14" s="37"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="37" t="s">
-        <v>124</v>
+      <c r="B15" s="38" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="36" t="s">
-        <v>125</v>
+      <c r="B16" s="37" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="36"/>
+      <c r="B17" s="37"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="37" t="s">
-        <v>126</v>
+      <c r="B18" s="38" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="36" t="s">
-        <v>127</v>
+      <c r="B19" s="37" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="36"/>
+      <c r="B20" s="37"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="37" t="s">
-        <v>128</v>
+      <c r="B21" s="38" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="36" t="s">
-        <v>129</v>
+      <c r="B22" s="37" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="36" t="s">
-        <v>130</v>
+      <c r="B23" s="37" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="36"/>
+      <c r="B24" s="37"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="37" t="s">
-        <v>131</v>
+      <c r="B25" s="38" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="36" t="s">
-        <v>132</v>
+      <c r="B26" s="37" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="36"/>
+      <c r="B27" s="37"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="37" t="s">
-        <v>133</v>
+      <c r="B28" s="38" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="36" t="s">
-        <v>134</v>
+      <c r="B29" s="37" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="36"/>
+      <c r="B30" s="37"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="37" t="s">
-        <v>135</v>
+      <c r="B31" s="38" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="36" t="s">
-        <v>136</v>
+      <c r="B32" s="37" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="36" t="s">
-        <v>137</v>
+      <c r="B33" s="37" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="36" t="s">
-        <v>138</v>
+      <c r="B34" s="37" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="36"/>
+      <c r="B35" s="37"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="37" t="s">
-        <v>139</v>
+      <c r="B36" s="38" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="36" t="s">
-        <v>140</v>
+      <c r="B37" s="37" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="36" t="s">
-        <v>141</v>
+      <c r="B38" s="37" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="36" t="s">
-        <v>142</v>
+      <c r="B39" s="37" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>